<commit_message>
BILAN-1 (avant merge, 1/4) — assiettes D.O / TRC recopiées du tableur : 0 € d'écart
Les assurances D.O / C.N.R et TRC + GAREAT ont, dans le modèle de la promotrice,
une assiette composée à la main : total (2) + étude de sol − imprévus (techniques).
On la reproduit à l'identique (plus de simplification « total (2) »).

- moteur : assiettes `total2_ttc_sol_imprevus` / `total2_ht_sol_imprevus` (étude
  de sol et imprévus calculés au staging) ; excel : mêmes formules composées.
- Non-régression : les 45 lignes au centime, 0 € d'écart ; résultat net du moteur
  = 1 244 996,78 € = le modèle ; « écran = PDF = Excel » tient toujours.
- Rapport §4 réécrit (0 écart), captures régénérées.

(Branche rebasée sans conflit sur e60bf578 — TUILES-TX-1 + VITESSE-PROD-1.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit-2026-10/bilan-1/captures/bilan-temoin.xlsx
+++ b/docs/audit-2026-10/bilan-1/captures/bilan-temoin.xlsx
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="B52" s="11">
-        <f>SUM(F34:F43)</f>
+        <f>SUM(F34:F43)+F25-F43</f>
         <v/>
       </c>
       <c r="C52" s="12" t="n">
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="B53" s="11">
-        <f>SUM(D34:D43)</f>
+        <f>SUM(D34:D43)+D25-D43</f>
         <v/>
       </c>
       <c r="C53" s="12" t="n">

</xml_diff>